<commit_message>
Update JISData sheet names for consistency and modify sample input Excel file.
</commit_message>
<xml_diff>
--- a/data/sample_input.xlsx
+++ b/data/sample_input.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11400" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="11400" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="01排产信息（输入）" sheetId="1" r:id="rId1"/>
-    <sheet name="02输入（SR拆分）" sheetId="2" r:id="rId2"/>
+    <sheet name="01排产信息 (输入)" sheetId="1" r:id="rId1"/>
+    <sheet name="02输入 (SR拆分)" sheetId="2" r:id="rId2"/>
     <sheet name="03包规基表" sheetId="3" r:id="rId3"/>
     <sheet name="04供应商作息&amp;车规基表" sheetId="4" r:id="rId4"/>
   </sheets>

</xml_diff>